<commit_message>
Match owned components and remove unnecessary breadboard rail bridges
</commit_message>
<xml_diff>
--- a/hardware-checklist.xlsx
+++ b/hardware-checklist.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="元件核对" sheetId="1" r:id="R39e96964ea034be1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="工具线材" sheetId="2" r:id="Rcb4cdde2e007421f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="元件核对" sheetId="1" r:id="R0e8ecd3a8b194b2e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="工具线材" sheetId="2" r:id="R495c7d2694754ffa"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -520,7 +520,7 @@
     </x:row>
     <x:row r="2" ht="30" customHeight="1">
       <x:c r="A2" s="3" t="str">
-        <x:v>节奏大师硬件核对清单（2026-10-14）</x:v>
+        <x:v>节奏大师硬件核对清单（2026-10-17）</x:v>
       </x:c>
       <x:c r="B2" s="2"/>
       <x:c r="C2" s="2"/>
@@ -558,7 +558,7 @@
     </x:row>
     <x:row r="4" ht="24" customHeight="1">
       <x:c r="A4" s="2" t="str">
-        <x:v>蓝色栏填写实物型号、已有数量和核对结果。设计用量留空表示需要按实际备料，不表示0。</x:v>
+        <x:v>蓝色栏填写实物型号、已有数量和核对结果。声音项目用量0表示当前未安装，待型号确认后重设计。</x:v>
       </x:c>
       <x:c r="B4" s="2"/>
       <x:c r="C4" s="2"/>
@@ -577,7 +577,7 @@
     </x:row>
     <x:row r="5" ht="24" customHeight="1">
       <x:c r="A5" s="2" t="str">
-        <x:v>两版共用元件可轮流使用一套；若要同时搭成两台，通用元件需另备一套。黄色型号是候选或尚未确认。</x:v>
+        <x:v>两版可轮流使用一套通用元件。已有三极管和蜂鸣器型号待核对，旧MOS预焊板方案已停用。</x:v>
       </x:c>
       <x:c r="B5" s="2"/>
       <x:c r="C5" s="2"/>
@@ -596,7 +596,7 @@
     </x:row>
     <x:row r="6" ht="24" customHeight="1">
       <x:c r="A6" s="2" t="str">
-        <x:v>13盏LED、6个按键。声音支路参数未定，请核对后再购买候选元件。</x:v>
+        <x:v>当前13盏LED、6个按键、OLED及供电。声音暂不接线，设计用量留空的项目按实际备料。</x:v>
       </x:c>
       <x:c r="B6" s="2"/>
       <x:c r="C6" s="2"/>
@@ -658,7 +658,7 @@
         <x:v>来源／型号参数参考</x:v>
       </x:c>
     </x:row>
-    <x:row r="8" ht="54" customHeight="1">
+    <x:row r="8" ht="68" customHeight="1">
       <x:c r="A8" s="24" t="str">
         <x:v>C01</x:v>
       </x:c>
@@ -670,7 +670,7 @@
       </x:c>
       <x:c r="D8" s="24" t="str">
         <x:v>使用现有板；3.3V逻辑；两侧各2×29扩展排针。
-控制13灯、6按键、OLED和声音。</x:v>
+控制灯和按键并连接OLED；声音接口暂留待设计。</x:v>
       </x:c>
       <x:c r="E8" s="25" t="n">
         <x:v>1</x:v>
@@ -697,7 +697,7 @@
       </x:c>
       <x:c r="N8" s="2"/>
       <x:c r="O8" s="5" t="str">
-        <x:v>Vishay原厂1N5817/18/19数据表，2026-10-14核对。
+        <x:v>旧声音候选参考，当前不安装。
 https://www.st.com/resource/en/datasheet/stm32f103ze.pdf</x:v>
       </x:c>
     </x:row>
@@ -838,7 +838,7 @@
         <x:v>通用轴向直插1kΩ；厂家及系列不限，现有型号未知</x:v>
       </x:c>
       <x:c r="D12" s="5" t="str">
-        <x:v>1kΩ（102），≥1/4W。每盏LED串联1只，共13只。与C06合计14只1kΩ电阻。</x:v>
+        <x:v>1kΩ（102），≥1/4W。每盏LED串联1只，本次共13只；声音电阻另行设计。</x:v>
       </x:c>
       <x:c r="E12" s="18" t="n">
         <x:v>13</x:v>
@@ -861,7 +861,7 @@
         <x:v>待核对</x:v>
       </x:c>
       <x:c r="M12" s="5" t="str">
-        <x:v>与C06合计14只使用，可准备20只含备用</x:v>
+        <x:v>只计算13只LED电阻；声音控制电阻待定，不再默认合计14只。</x:v>
       </x:c>
       <x:c r="N12" s="2"/>
       <x:c r="O12" s="5" t="str">
@@ -873,28 +873,28 @@
         <x:v>C06</x:v>
       </x:c>
       <x:c r="B13" s="24" t="str">
-        <x:v>MOS栅极串联电阻</x:v>
-      </x:c>
-      <x:c r="C13" s="24" t="str">
-        <x:v>通用轴向直插1kΩ；与LED电阻可同规格</x:v>
+        <x:v>停用的旧MOS控制电阻</x:v>
+      </x:c>
+      <x:c r="C13" s="29" t="str">
+        <x:v>旧候选1kΩ；当前不安装</x:v>
       </x:c>
       <x:c r="D13" s="24" t="str">
-        <x:v>1kΩ（102），≥1/4W。声音MOS的G脚前串联1只。与C05合计14只，不能漏算。</x:v>
+        <x:v>旧MOS栅极1kΩ控制电阻已停用，不适用于直接套接现有三极管。新控制电阻在型号确认后设计。</x:v>
       </x:c>
       <x:c r="E13" s="25" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="F13" s="24" t="str">
-        <x:v>只</x:v>
+        <x:v>只（当前安装）</x:v>
       </x:c>
       <x:c r="G13" s="24" t="str">
-        <x:v>两版采用当前MOS声音方案时</x:v>
+        <x:v>两版当前均暂停</x:v>
       </x:c>
       <x:c r="H13" s="24" t="str">
         <x:v>用户有1kΩ；数量待清点</x:v>
       </x:c>
       <x:c r="I13" s="24" t="str">
-        <x:v>声音采用MOS候选时才计入；若另选NPN方案，应重新核算，不可直接照换。</x:v>
+        <x:v>不能把旧MOS栅极电阻直接当三极管基极电阻。</x:v>
       </x:c>
       <x:c r="J13" s="26"/>
       <x:c r="K13" s="27"/>
@@ -902,7 +902,7 @@
         <x:v>待核对</x:v>
       </x:c>
       <x:c r="M13" s="24" t="str">
-        <x:v>已计入1kΩ合计14只，避免重复统计</x:v>
+        <x:v>暂停安装，驱动定型后确认新阻值。</x:v>
       </x:c>
       <x:c r="N13" s="2"/>
       <x:c r="O13" s="5" t="str">
@@ -1038,29 +1038,29 @@
         <x:v>C10</x:v>
       </x:c>
       <x:c r="B17" s="24" t="str">
-        <x:v>两脚无源发声器／蜂鸣器</x:v>
+        <x:v>现有蜂鸣器（未接线）</x:v>
       </x:c>
       <x:c r="C17" s="29" t="str">
-        <x:v>现有具体型号未知；赛题清单标16Ω</x:v>
+        <x:v>实物型号未知，等待核对</x:v>
       </x:c>
       <x:c r="D17" s="24" t="str">
-        <x:v>无源和磁性类型仍需确认；16Ω不是额定电压、功率或允许长期直流的证明。
-播放比赛音符。</x:v>
+        <x:v>用户确认有1件。赛题材料列16Ω；类型和额定参数待确认。
+比赛按键发声和旋律演奏使用，当前未安装。</x:v>
       </x:c>
       <x:c r="E17" s="25" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="F17" s="24" t="str">
-        <x:v>个</x:v>
+        <x:v>个（当前安装）</x:v>
       </x:c>
       <x:c r="G17" s="24" t="str">
-        <x:v>洞洞板、面包板共用</x:v>
+        <x:v>两版共用，声音待设计</x:v>
       </x:c>
       <x:c r="H17" s="24" t="str">
-        <x:v>已有底部照片及正极标志；额定参数未知</x:v>
+        <x:v>已有1个，2026-10-17确认；型号未知。</x:v>
       </x:c>
       <x:c r="I17" s="24" t="str">
-        <x:v>确认型号、无源／有源、额定电压、电流、类型、极性及脚距；不能直接接GPIO。</x:v>
+        <x:v>核对完整型号、类型、额定电压/电流、极性及脚距；禁止直接接GPIO。</x:v>
       </x:c>
       <x:c r="J17" s="26"/>
       <x:c r="K17" s="27"/>
@@ -1068,40 +1068,40 @@
         <x:v>待核对</x:v>
       </x:c>
       <x:c r="M17" s="24" t="str">
-        <x:v>先核对现有1个；清单2个不是已确认库存</x:v>
+        <x:v>已有1个保留待装；型号确认前不接线、不补购未知型号。</x:v>
       </x:c>
       <x:c r="N17" s="2"/>
       <x:c r="O17" s="5" t="str">
-        <x:v>赛题材料清单、用户照片或已确认回复、当前两版接线设计</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="18" ht="68" customHeight="1">
+        <x:v>赛题材料清单、用户2026-10-17确认回复</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="54" customHeight="1">
       <x:c r="A18" s="5" t="str">
         <x:v>C11</x:v>
       </x:c>
       <x:c r="B18" s="5" t="str">
-        <x:v>逻辑电平N沟道MOS预焊转接板</x:v>
+        <x:v>现有三极管（未接线）</x:v>
       </x:c>
       <x:c r="C18" s="28" t="str">
-        <x:v>候选AO3400A预焊板；不是裸SOT-23贴片管</x:v>
+        <x:v>用户已有，型号稍后提供</x:v>
       </x:c>
       <x:c r="D18" s="5" t="str">
-        <x:v>候选AO3400A预焊转接板，带G/D/S端子。芯片为30V N-MOS，VGS=2.5V时RDS(on)最大48mΩ。用于3.3V信号控制声音支路，成品板脚序需另核对。</x:v>
+        <x:v>已有三极管，型号稍后提供。器件类型、封装、额定及B/C/E脚序待核对，不能假定NPN/PNP/TO-92；目前未接线。</x:v>
       </x:c>
       <x:c r="E18" s="18" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="F18" s="5" t="str">
-        <x:v>块</x:v>
+        <x:v>个（当前安装）</x:v>
       </x:c>
       <x:c r="G18" s="5" t="str">
-        <x:v>两版采用当前MOS声音方案时</x:v>
+        <x:v>两版共用，驱动待设计</x:v>
       </x:c>
       <x:c r="H18" s="5" t="str">
-        <x:v>未确认已有；不能写成已拥有</x:v>
+        <x:v>已有三极管，型号稍后提供、数量待清点；没有MOS预焊板。</x:v>
       </x:c>
       <x:c r="I18" s="5" t="str">
-        <x:v>购买前核对预焊、端子脚序、原理图、板载元件及3.3V控制能力；模型G-D-S顺序不是商品保证脚序。</x:v>
+        <x:v>提供完整型号和厂家信息，核对类型、额定值及真实B/C/E脚序；不能套用旧G/D/S。</x:v>
       </x:c>
       <x:c r="J18" s="21"/>
       <x:c r="K18" s="22"/>
@@ -1109,50 +1109,49 @@
         <x:v>待核对</x:v>
       </x:c>
       <x:c r="M18" s="5" t="str">
-        <x:v>确认发声器及具体模块后选1块</x:v>
+        <x:v>先核对现物型号及适用性，不要求AO3400A预焊板。</x:v>
       </x:c>
       <x:c r="N18" s="2"/>
       <x:c r="O18" s="5" t="str">
-        <x:v>AOS原厂AO3400A参数，2026-10-14核对。
-https://www.aosmd.com/products/mosfets/low-voltage-mosfets-12v-30v/ao3400a</x:v>
+        <x:v>用户2026-10-17确认回复</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="54" customHeight="1">
-      <x:c r="A19" s="5" t="str">
+      <x:c r="A19" s="24" t="str">
         <x:v>C12</x:v>
       </x:c>
-      <x:c r="B19" s="5" t="str">
-        <x:v>MOS栅极下拉电阻</x:v>
-      </x:c>
-      <x:c r="C19" s="5" t="str">
-        <x:v>通用轴向直插100kΩ</x:v>
-      </x:c>
-      <x:c r="D19" s="5" t="str">
-        <x:v>100kΩ（104）；≥1/4W。电阻104与陶瓷电容104的单位不同。
-G脚下拉到GND，帮助复位时关闭MOS。</x:v>
-      </x:c>
-      <x:c r="E19" s="18" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F19" s="5" t="str">
-        <x:v>只</x:v>
-      </x:c>
-      <x:c r="G19" s="5" t="str">
-        <x:v>两版采用当前MOS声音方案时</x:v>
-      </x:c>
-      <x:c r="H19" s="5" t="str">
+      <x:c r="B19" s="24" t="str">
+        <x:v>待定的声音驱动下拉电阻</x:v>
+      </x:c>
+      <x:c r="C19" s="29" t="str">
+        <x:v>旧候选100kΩ；当前不安装</x:v>
+      </x:c>
+      <x:c r="D19" s="24" t="str">
+        <x:v>旧MOS方案采用100kΩ下拉；三极管驱动定型后重新确定。
+新声音支路设计后确定。</x:v>
+      </x:c>
+      <x:c r="E19" s="25" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F19" s="24" t="str">
+        <x:v>只（当前安装）</x:v>
+      </x:c>
+      <x:c r="G19" s="24" t="str">
+        <x:v>两版当前均暂停</x:v>
+      </x:c>
+      <x:c r="H19" s="24" t="str">
         <x:v>未确认；用户仅明确有1kΩ和10kΩ</x:v>
       </x:c>
-      <x:c r="I19" s="5" t="str">
-        <x:v>确认阻值与库存。</x:v>
-      </x:c>
-      <x:c r="J19" s="21"/>
-      <x:c r="K19" s="22"/>
-      <x:c r="L19" s="21" t="str">
-        <x:v>待核对</x:v>
-      </x:c>
-      <x:c r="M19" s="5" t="str">
-        <x:v>1只使用，库存先清点</x:v>
+      <x:c r="I19" s="24" t="str">
+        <x:v>当前0表示暂不安装；比赛最终仍需声音及相应保护。</x:v>
+      </x:c>
+      <x:c r="J19" s="26"/>
+      <x:c r="K19" s="27"/>
+      <x:c r="L19" s="26" t="str">
+        <x:v>待核对</x:v>
+      </x:c>
+      <x:c r="M19" s="24" t="str">
+        <x:v>暂停安装，不按旧候选值默认购买。</x:v>
       </x:c>
       <x:c r="N19" s="2"/>
       <x:c r="O19" s="5" t="str">
@@ -1164,29 +1163,29 @@
         <x:v>C13</x:v>
       </x:c>
       <x:c r="B20" s="5" t="str">
-        <x:v>声音限流功率电阻</x:v>
+        <x:v>待定的声音限流功率电阻</x:v>
       </x:c>
       <x:c r="C20" s="28" t="str">
-        <x:v>候选68Ω，≥1W轴向直插</x:v>
+        <x:v>旧候选68Ω、≥1W；当前不安装</x:v>
       </x:c>
       <x:c r="D20" s="5" t="str">
-        <x:v>68Ω；≥1W；候选按±5%或更好；不是普通1/4W同阻值电阻。
-串联在声音电源与发声器正端之间。</x:v>
+        <x:v>需按现有蜂鸣器额定参数和实测供电重定，不默认保留68Ω。
+新声音支路设计后确定。</x:v>
       </x:c>
       <x:c r="E20" s="18" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="F20" s="5" t="str">
-        <x:v>只</x:v>
+        <x:v>只（当前安装）</x:v>
       </x:c>
       <x:c r="G20" s="5" t="str">
-        <x:v>两版当前5V声音支路候选</x:v>
+        <x:v>两版当前均暂停</x:v>
       </x:c>
       <x:c r="H20" s="5" t="str">
         <x:v>未确认</x:v>
       </x:c>
       <x:c r="I20" s="5" t="str">
-        <x:v>4.5V与5V、发声器额定电流不同会影响选择；当前不是最终值，不能省略或短接。</x:v>
+        <x:v>当前0表示暂不安装；比赛最终仍需声音及相应保护。</x:v>
       </x:c>
       <x:c r="J20" s="21"/>
       <x:c r="K20" s="22"/>
@@ -1194,7 +1193,7 @@
         <x:v>待核对</x:v>
       </x:c>
       <x:c r="M20" s="5" t="str">
-        <x:v>发声器与供电确认后再定值和采购</x:v>
+        <x:v>暂停安装，不按旧候选值默认购买。</x:v>
       </x:c>
       <x:c r="N20" s="2"/>
       <x:c r="O20" s="5" t="str">
@@ -1206,29 +1205,29 @@
         <x:v>C14</x:v>
       </x:c>
       <x:c r="B21" s="5" t="str">
-        <x:v>声音保护二极管</x:v>
+        <x:v>待定的声音保护二极管</x:v>
       </x:c>
       <x:c r="C21" s="28" t="str">
-        <x:v>候选1N5819肖特基轴向直插</x:v>
+        <x:v>旧候选1N5819；当前不安装</x:v>
       </x:c>
       <x:c r="D21" s="5" t="str">
-        <x:v>1A、40V额定；若确认为电磁线圈，K端跨接发声器正端，A端跨接开关负端。
-为线圈关断时的电流提供回路。</x:v>
+        <x:v>用户有二极管但型号未知；先确认蜂鸣器类型和驱动，再定保护器件。
+新声音支路设计后确定。</x:v>
       </x:c>
       <x:c r="E21" s="18" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="F21" s="5" t="str">
-        <x:v>只</x:v>
+        <x:v>只（当前安装）</x:v>
       </x:c>
       <x:c r="G21" s="5" t="str">
-        <x:v>两版电磁发声器驱动候选</x:v>
+        <x:v>两版当前均暂停</x:v>
       </x:c>
       <x:c r="H21" s="5" t="str">
         <x:v>用户说有二极管；具体型号与数量未知</x:v>
       </x:c>
       <x:c r="I21" s="5" t="str">
-        <x:v>核对1N5819型号、K端色环和方向；普通未知二极管不自动视作等效。</x:v>
+        <x:v>当前0表示暂不安装；比赛最终仍需声音及相应保护。</x:v>
       </x:c>
       <x:c r="J21" s="21"/>
       <x:c r="K21" s="22"/>
@@ -1236,11 +1235,11 @@
         <x:v>待核对</x:v>
       </x:c>
       <x:c r="M21" s="5" t="str">
-        <x:v>先查现有型号，合适则不必再买</x:v>
+        <x:v>暂停安装，不按旧候选值默认购买。</x:v>
       </x:c>
       <x:c r="N21" s="2"/>
       <x:c r="O21" s="5" t="str">
-        <x:v>Vishay原厂1N5817/18/19数据表，2026-10-14核对。
+        <x:v>旧声音候选参考，当前不安装。
 https://www.vishay.com/docs/88525/1n5817.pdf</x:v>
       </x:c>
     </x:row>
@@ -1249,29 +1248,29 @@
         <x:v>C15</x:v>
       </x:c>
       <x:c r="B22" s="5" t="str">
-        <x:v>陶瓷去耦电容</x:v>
-      </x:c>
-      <x:c r="C22" s="5" t="str">
-        <x:v>通用100nF（0.1µF，104）直插陶瓷</x:v>
+        <x:v>待定的声音去耦陶瓷电容</x:v>
+      </x:c>
+      <x:c r="C22" s="28" t="str">
+        <x:v>旧候选100nF（104）；当前不安装</x:v>
       </x:c>
       <x:c r="D22" s="5" t="str">
-        <x:v>100nF；耐压≥16V；无极性。
-声音电源与GND之间的高频去耦。</x:v>
+        <x:v>驱动和供电定型后确认容量、耐压和安装位置。
+新声音支路设计后确定。</x:v>
       </x:c>
       <x:c r="E22" s="18" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="F22" s="5" t="str">
-        <x:v>只</x:v>
+        <x:v>只（当前安装）</x:v>
       </x:c>
       <x:c r="G22" s="5" t="str">
-        <x:v>两版声音支路候选</x:v>
+        <x:v>两版当前均暂停</x:v>
       </x:c>
       <x:c r="H22" s="5" t="str">
         <x:v>用户说电容可以买，现有库存未确认</x:v>
       </x:c>
       <x:c r="I22" s="5" t="str">
-        <x:v>核对容量、耐压和脚距；不要把104电容认作100kΩ电阻。</x:v>
+        <x:v>当前0表示暂不安装；比赛最终仍需声音及相应保护。</x:v>
       </x:c>
       <x:c r="J22" s="21"/>
       <x:c r="K22" s="22"/>
@@ -1279,7 +1278,7 @@
         <x:v>待核对</x:v>
       </x:c>
       <x:c r="M22" s="5" t="str">
-        <x:v>1只使用，可备2～5只</x:v>
+        <x:v>暂停安装，不按旧候选值默认购买。</x:v>
       </x:c>
       <x:c r="N22" s="2"/>
       <x:c r="O22" s="5" t="str">
@@ -1291,29 +1290,29 @@
         <x:v>C16</x:v>
       </x:c>
       <x:c r="B23" s="5" t="str">
-        <x:v>电解储能电容</x:v>
-      </x:c>
-      <x:c r="C23" s="5" t="str">
-        <x:v>通用100µF径向直插铝电解</x:v>
+        <x:v>待定的声音电解电容</x:v>
+      </x:c>
+      <x:c r="C23" s="28" t="str">
+        <x:v>旧候选100µF；当前不安装</x:v>
       </x:c>
       <x:c r="D23" s="5" t="str">
-        <x:v>100µF；耐压≥16V；有正负极。
-声音电源与GND之间缓冲短时负载变化。</x:v>
+        <x:v>驱动和供电定型后确认容量、耐压、极性和安装位置。
+新声音支路设计后确定。</x:v>
       </x:c>
       <x:c r="E23" s="18" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="F23" s="5" t="str">
-        <x:v>只</x:v>
+        <x:v>只（当前安装）</x:v>
       </x:c>
       <x:c r="G23" s="5" t="str">
-        <x:v>两版声音支路候选</x:v>
+        <x:v>两版当前均暂停</x:v>
       </x:c>
       <x:c r="H23" s="5" t="str">
         <x:v>可购买，库存未确认</x:v>
       </x:c>
       <x:c r="I23" s="5" t="str">
-        <x:v>确认100µF与≥16V均满足；外壳负极条纹接GND；实际脚距与模型需适配。</x:v>
+        <x:v>当前0表示暂不安装；比赛最终仍需声音及相应保护。</x:v>
       </x:c>
       <x:c r="J23" s="21"/>
       <x:c r="K23" s="22"/>
@@ -1321,7 +1320,7 @@
         <x:v>待核对</x:v>
       </x:c>
       <x:c r="M23" s="5" t="str">
-        <x:v>1只使用，可备2只</x:v>
+        <x:v>暂停安装，不按旧候选值默认购买。</x:v>
       </x:c>
       <x:c r="N23" s="2"/>
       <x:c r="O23" s="5" t="str">
@@ -1501,29 +1500,29 @@
         <x:v>P05</x:v>
       </x:c>
       <x:c r="B28" s="5" t="str">
-        <x:v>声音支路电源／发声器接口排针</x:v>
+        <x:v>暂停的声音支路接口排针</x:v>
       </x:c>
       <x:c r="C28" s="5" t="str">
         <x:v>通用2.54mm单排1×2排针</x:v>
       </x:c>
       <x:c r="D28" s="5" t="str">
-        <x:v>J_POWER 1段＋J_BUZZ 1段；共4针。
-一段接核心板取出的声音电源与地；一段接发声器两端。</x:v>
+        <x:v>旧J_POWER与J_BUZZ各2针，当前均不安装；新驱动设计后重定接口。
+历史声音接口记录。</x:v>
       </x:c>
       <x:c r="E28" s="18" t="n">
-        <x:v>2</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="F28" s="5" t="str">
-        <x:v>段</x:v>
+        <x:v>段（当前安装）</x:v>
       </x:c>
       <x:c r="G28" s="5" t="str">
-        <x:v>洞洞板采用声音候选支路时</x:v>
+        <x:v>洞洞板声音定型后确认</x:v>
       </x:c>
       <x:c r="H28" s="5" t="str">
         <x:v>有排针或排母，数量未确认</x:v>
       </x:c>
       <x:c r="I28" s="5" t="str">
-        <x:v>不是充电宝上的分线接头；声音支路5V取电仍待测。两接口功能与极性不同。</x:v>
+        <x:v>这不表示充电宝需要分线、第二条线或额外电源模块。</x:v>
       </x:c>
       <x:c r="J28" s="21"/>
       <x:c r="K28" s="22"/>
@@ -1531,7 +1530,7 @@
         <x:v>待核对</x:v>
       </x:c>
       <x:c r="M28" s="5" t="str">
-        <x:v>可由40针长条各裁成2针</x:v>
+        <x:v>暂停旧2段接头，不作为本次必购项。</x:v>
       </x:c>
       <x:c r="N28" s="2"/>
       <x:c r="O28" s="5" t="str">
@@ -1588,8 +1587,8 @@
         <x:v>MB-102；用户照片同型两块</x:v>
       </x:c>
       <x:c r="D30" s="24" t="str">
-        <x:v>每块中央a～j、编号1～63；模型电源条按上下半段绘制，实物通断需测。
-第一块轨1／2与控制／OLED，第二块轨3／4与声音候选区域。</x:v>
+        <x:v>每块中央a～j、编号1～63。当前只从电源条前半段取电，不装中点桥接。
+第一块轨1/2、控制与OLED，第二块轨3/4；声音配套暂停。</x:v>
       </x:c>
       <x:c r="E30" s="25" t="n">
         <x:v>2</x:v>
@@ -1604,7 +1603,7 @@
         <x:v>用户明确有2块，已给照片</x:v>
       </x:c>
       <x:c r="I30" s="24" t="str">
-        <x:v>确认五孔同组导通、中央沟槽隔离、电源条是否分段；若与模型不同，先适配。</x:v>
+        <x:v>断电测五孔同组、电源条前半段导通和沟槽隔离；后半段当前不取电，不默认需要跨中点线。</x:v>
       </x:c>
       <x:c r="J30" s="26"/>
       <x:c r="K30" s="27"/>
@@ -1630,11 +1629,11 @@
         <x:v>2.54mm公对公杜邦线或适配面包板的实芯短跳线</x:v>
       </x:c>
       <x:c r="D31" s="5" t="str">
-        <x:v>两端为金属针；连接面包板插孔。不同颜色，长度按实际布局。
-板内信号、共地、跨板电源和电源条跨断点连接。</x:v>
+        <x:v>两端金属针。当前29根，可选I²C上拉另加2根；不含旧声音线和5根已撤桥线。
+板内信号、公共地和两板电源连接，电源条只取前半段。</x:v>
       </x:c>
       <x:c r="E31" s="18" t="n">
-        <x:v>38</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="F31" s="5" t="str">
         <x:v>根（当前计划）</x:v>
@@ -1646,7 +1645,7 @@
         <x:v>用户有杜邦线；公公类型和数量待清点</x:v>
       </x:c>
       <x:c r="I31" s="5" t="str">
-        <x:v>38为代码计划中非可选公公连接计数，不是全部跳线总数；MOS模块适配按实物另计。</x:v>
+        <x:v>29是新版公公连接数量，不是全部跳线数；声音定型后追加，不沿用旧38根。</x:v>
       </x:c>
       <x:c r="J31" s="21"/>
       <x:c r="K31" s="22"/>
@@ -1654,7 +1653,7 @@
         <x:v>待核对</x:v>
       </x:c>
       <x:c r="M31" s="5" t="str">
-        <x:v>当前非可选连接约38根，可先清点40根以上；可选上拉另加2根</x:v>
+        <x:v>清点29根，线长按实际布局；可选上拉需要时再加2根。</x:v>
       </x:c>
       <x:c r="N31" s="2"/>
       <x:c r="O31" s="5" t="str">
@@ -1672,11 +1671,11 @@
         <x:v>2.54mm公对母，长度按核心板到面包板／模块距离</x:v>
       </x:c>
       <x:c r="D32" s="5" t="str">
-        <x:v>一端金属针，另一端插孔；不强求旧清单10cm，较长连接可用20～40cm级。
+        <x:v>一端金属针、另一端插孔。核心板23根加OLED4根，共27根，已排除声音支路。
 核心板排针／OLED排针连接面包板。</x:v>
       </x:c>
       <x:c r="E32" s="18" t="n">
-        <x:v>30</x:v>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="F32" s="5" t="str">
         <x:v>根（当前计划）</x:v>
@@ -1688,7 +1687,7 @@
         <x:v>用户有杜邦线；公母类型和数量待清点</x:v>
       </x:c>
       <x:c r="I32" s="5" t="str">
-        <x:v>模块端要有可靠排针；线长按布局，MOS实际脚序未核对前不照图插。</x:v>
+        <x:v>27按模块已有公排针计算，接头改变需适配；旧MOS模块适配线不再计入。</x:v>
       </x:c>
       <x:c r="J32" s="21"/>
       <x:c r="K32" s="22"/>
@@ -1696,7 +1695,7 @@
         <x:v>待核对</x:v>
       </x:c>
       <x:c r="M32" s="5" t="str">
-        <x:v>当前核心板26根＋OLED4根约30根；MOS板外适配约3根另计，可清点40根含余量</x:v>
+        <x:v>清点27根，线长按核心板、面包板和OLED实际距离。</x:v>
       </x:c>
       <x:c r="N32" s="2"/>
       <x:c r="O32" s="5" t="str">
@@ -1760,7 +1759,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra7ba55bacf214ade"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0430a476cb6e495d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1808,7 +1807,7 @@
     </x:row>
     <x:row r="2" ht="30" customHeight="1">
       <x:c r="A2" s="3" t="str">
-        <x:v>节奏大师工具、线材与选件（2026-10-14）</x:v>
+        <x:v>节奏大师工具、线材与选件（2026-10-17）</x:v>
       </x:c>
       <x:c r="B2" s="2"/>
       <x:c r="C2" s="2"/>
@@ -1846,7 +1845,7 @@
     </x:row>
     <x:row r="4" ht="24" customHeight="1">
       <x:c r="A4" s="2" t="str">
-        <x:v>蓝色栏填写实物型号、已有数量和核对结果。设计用量留空表示需要按实际备料，不表示0。</x:v>
+        <x:v>蓝色栏填写实物型号、已有数量和核对结果。声音项目用量0表示当前未安装，待型号确认后重设计。</x:v>
       </x:c>
       <x:c r="B4" s="2"/>
       <x:c r="C4" s="2"/>
@@ -1865,7 +1864,7 @@
     </x:row>
     <x:row r="5" ht="24" customHeight="1">
       <x:c r="A5" s="2" t="str">
-        <x:v>两版共用元件可轮流使用一套；若要同时搭成两台，通用元件需另备一套。黄色型号是候选或尚未确认。</x:v>
+        <x:v>两版可轮流使用一套通用元件。已有三极管和蜂鸣器型号待核对，旧MOS预焊板方案已停用。</x:v>
       </x:c>
       <x:c r="B5" s="2"/>
       <x:c r="C5" s="2"/>
@@ -1884,7 +1883,7 @@
     </x:row>
     <x:row r="6" ht="24" customHeight="1">
       <x:c r="A6" s="2" t="str">
-        <x:v>先清点已有工具。W03是接口排针的汇总备料说明，不与P02～P05、W01重复相加。</x:v>
+        <x:v>当前公公29根、公母27根及成品线1条；可选上拉另加2根公公。W03汇总P02～P04、W01，不重复备料。</x:v>
       </x:c>
       <x:c r="B6" s="2"/>
       <x:c r="C6" s="2"/>
@@ -2021,7 +2020,7 @@
         <x:v>待核对</x:v>
       </x:c>
       <x:c r="M9" s="5" t="str">
-        <x:v>洞洞板版按13灯信号＋6键信号＋3V3/GND＋OLED／声音接口清点，40根一排可作为备料参考</x:v>
+        <x:v>按13灯信号、6键信号、3V3/GND及OLED接头清点；声音接口暂不计入。</x:v>
       </x:c>
       <x:c r="N9" s="2"/>
       <x:c r="O9" s="5" t="str">
@@ -2039,7 +2038,7 @@
         <x:v>通用40针可裁单排排针；排母按实际选用</x:v>
       </x:c>
       <x:c r="D10" s="5" t="str">
-        <x:v>洞洞板接口共29针＋OLED自身4针（若未焊）；核心板116针已装。
+        <x:v>当前洞洞板接口25针，加OLED自身4针（若未焊）合计29针；核心板116针已装。
 裁成各接口所需针数。</x:v>
       </x:c>
       <x:c r="E10" s="18"/>
@@ -2053,7 +2052,7 @@
         <x:v>用户确认有排针或排母，规格与长度数量待清点</x:v>
       </x:c>
       <x:c r="I10" s="5" t="str">
-        <x:v>确认实际是排针还是排母，针距和剪裁损耗；不再给核心板重复采购整套排针。</x:v>
+        <x:v>确认排针/排母、针距和裁切损耗；不重复采购核心板排针，声音定型后再追加。</x:v>
       </x:c>
       <x:c r="J10" s="21"/>
       <x:c r="K10" s="22"/>
@@ -2061,7 +2060,7 @@
         <x:v>待核对</x:v>
       </x:c>
       <x:c r="M10" s="5" t="str">
-        <x:v>本行是P02～P05与W01的汇总备料，不应再叠加采购用量；40针长条1条理论可裁33针，裁切损耗／备用另计</x:v>
+        <x:v>汇总P02～P04与W01，不重复相加。40针长条1条理论可裁29针，损耗及备用另计；停用P05不计。</x:v>
       </x:c>
       <x:c r="N10" s="2"/>
       <x:c r="O10" s="5" t="str">
@@ -2456,7 +2455,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re1985030f2744156"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0d9507e6e9734120"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Confirm owned passive 16-ohm buzzer specification
</commit_message>
<xml_diff>
--- a/hardware-checklist.xlsx
+++ b/hardware-checklist.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="元件核对" sheetId="1" r:id="R0e8ecd3a8b194b2e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="工具线材" sheetId="2" r:id="R495c7d2694754ffa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="元件核对" sheetId="1" r:id="Rcb47f9536eb647b8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="工具线材" sheetId="2" r:id="R54584589b20a4932"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1038,14 +1038,14 @@
         <x:v>C10</x:v>
       </x:c>
       <x:c r="B17" s="24" t="str">
-        <x:v>现有蜂鸣器（未接线）</x:v>
+        <x:v>现有无源蜂鸣器（未接线）</x:v>
       </x:c>
       <x:c r="C17" s="29" t="str">
-        <x:v>实物型号未知，等待核对</x:v>
+        <x:v>型号未知（无源、16Ω已确认）</x:v>
       </x:c>
       <x:c r="D17" s="24" t="str">
-        <x:v>用户确认有1件。赛题材料列16Ω；类型和额定参数待确认。
-比赛按键发声和旋律演奏使用，当前未安装。</x:v>
+        <x:v>用户2026-10-17确认：无源、16Ω。额定电压/电流及端子定义待确认。
+用于比赛按键发声和旋律演奏，当前未安装。</x:v>
       </x:c>
       <x:c r="E17" s="25" t="n">
         <x:v>0</x:v>
@@ -1057,10 +1057,10 @@
         <x:v>两版共用，声音待设计</x:v>
       </x:c>
       <x:c r="H17" s="24" t="str">
-        <x:v>已有1个，2026-10-17确认；型号未知。</x:v>
+        <x:v>已有1个无源蜂鸣器，16Ω。2026-10-17用户确认，具体型号未知。</x:v>
       </x:c>
       <x:c r="I17" s="24" t="str">
-        <x:v>核对完整型号、类型、额定电压/电流、极性及脚距；禁止直接接GPIO。</x:v>
+        <x:v>核对完整型号、额定电压/电流、实物端子定义及脚距；禁止直接接GPIO。</x:v>
       </x:c>
       <x:c r="J17" s="26"/>
       <x:c r="K17" s="27"/>
@@ -1068,11 +1068,11 @@
         <x:v>待核对</x:v>
       </x:c>
       <x:c r="M17" s="24" t="str">
-        <x:v>已有1个保留待装；型号确认前不接线、不补购未知型号。</x:v>
+        <x:v>已有1个保留待装；待额定参数和三极管型号、脚序确认后设计接线，不补购未知型号。</x:v>
       </x:c>
       <x:c r="N17" s="2"/>
       <x:c r="O17" s="5" t="str">
-        <x:v>赛题材料清单、用户2026-10-17确认回复</x:v>
+        <x:v>用户2026-10-17确认：无源蜂鸣器，16Ω；具体型号和额定参数未提供。</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="54" customHeight="1">
@@ -1211,7 +1211,7 @@
         <x:v>旧候选1N5819；当前不安装</x:v>
       </x:c>
       <x:c r="D21" s="5" t="str">
-        <x:v>用户有二极管但型号未知；先确认蜂鸣器类型和驱动，再定保护器件。
+        <x:v>用户有二极管但型号未知。蜂鸣器已确认无源、16Ω；额定参数和三极管驱动确定后，再定保护器件。
 新声音支路设计后确定。</x:v>
       </x:c>
       <x:c r="E21" s="18" t="n">
@@ -1759,7 +1759,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0430a476cb6e495d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc321b6af3ec54baf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2455,7 +2455,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0d9507e6e9734120"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4acc825996db4c8f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Fix switch clearance and model purchased BJT buzzer trial in both layouts
</commit_message>
<xml_diff>
--- a/hardware-checklist.xlsx
+++ b/hardware-checklist.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="元件核对" sheetId="1" r:id="Rcb47f9536eb647b8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="工具线材" sheetId="2" r:id="R54584589b20a4932"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="元件核对" sheetId="1" r:id="R3f529c4e737747b3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="工具线材" sheetId="2" r:id="Re31429ef414b4ef6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -520,7 +520,7 @@
     </x:row>
     <x:row r="2" ht="30" customHeight="1">
       <x:c r="A2" s="3" t="str">
-        <x:v>节奏大师硬件核对清单（2026-10-17）</x:v>
+        <x:v>节奏大师硬件核对清单（2026-10-18）</x:v>
       </x:c>
       <x:c r="B2" s="2"/>
       <x:c r="C2" s="2"/>
@@ -558,7 +558,7 @@
     </x:row>
     <x:row r="4" ht="24" customHeight="1">
       <x:c r="A4" s="2" t="str">
-        <x:v>蓝色栏填写实物型号、已有数量和核对结果。声音项目用量0表示当前未安装，待型号确认后重设计。</x:v>
+        <x:v>蓝色栏填写实物型号、已有数量和核对结果。声音用量为采购后试接计划，尚未实物验收。</x:v>
       </x:c>
       <x:c r="B4" s="2"/>
       <x:c r="C4" s="2"/>
@@ -577,7 +577,7 @@
     </x:row>
     <x:row r="5" ht="24" customHeight="1">
       <x:c r="A5" s="2" t="str">
-        <x:v>两版可轮流使用一套通用元件。已有三极管和蜂鸣器型号待核对，旧MOS预焊板方案已停用。</x:v>
+        <x:v>两版共用元件。沿用现有无源16Ω蜂鸣器，SS8050D三极管待购；旧MOS转接板不使用。</x:v>
       </x:c>
       <x:c r="B5" s="2"/>
       <x:c r="C5" s="2"/>
@@ -596,7 +596,7 @@
     </x:row>
     <x:row r="6" ht="24" customHeight="1">
       <x:c r="A6" s="2" t="str">
-        <x:v>当前13盏LED、6个按键、OLED及供电。声音暂不接线，设计用量留空的项目按实际备料。</x:v>
+        <x:v>13盏LED、6个按键、OLED与充电宝供电；新增SS8050D限流试接支路，正式声音参数待测。</x:v>
       </x:c>
       <x:c r="B6" s="2"/>
       <x:c r="C6" s="2"/>
@@ -861,7 +861,7 @@
         <x:v>待核对</x:v>
       </x:c>
       <x:c r="M12" s="5" t="str">
-        <x:v>只计算13只LED电阻；声音控制电阻待定，不再默认合计14只。</x:v>
+        <x:v>LED用13只；声音基极另用2只1kΩ，合计至少15只。</x:v>
       </x:c>
       <x:c r="N12" s="2"/>
       <x:c r="O12" s="5" t="str">
@@ -873,28 +873,28 @@
         <x:v>C06</x:v>
       </x:c>
       <x:c r="B13" s="24" t="str">
-        <x:v>停用的旧MOS控制电阻</x:v>
+        <x:v>声音基极电阻（两只并联）</x:v>
       </x:c>
       <x:c r="C13" s="29" t="str">
-        <x:v>旧候选1kΩ；当前不安装</x:v>
+        <x:v>通用1kΩ轴向直插，两只并联等效500Ω</x:v>
       </x:c>
       <x:c r="D13" s="24" t="str">
-        <x:v>旧MOS栅极1kΩ控制电阻已停用，不适用于直接套接现有三极管。新控制电阻在型号确认后设计。</x:v>
+        <x:v>每只≥1/4W。PB0经两只并联电阻接SS8050D的B脚。</x:v>
       </x:c>
       <x:c r="E13" s="25" t="n">
-        <x:v>0</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="F13" s="24" t="str">
-        <x:v>只（当前安装）</x:v>
+        <x:v>只（计划）</x:v>
       </x:c>
       <x:c r="G13" s="24" t="str">
-        <x:v>两版当前均暂停</x:v>
+        <x:v>两版声音试接共用</x:v>
       </x:c>
       <x:c r="H13" s="24" t="str">
         <x:v>用户有1kΩ；数量待清点</x:v>
       </x:c>
       <x:c r="I13" s="24" t="str">
-        <x:v>不能把旧MOS栅极电阻直接当三极管基极电阻。</x:v>
+        <x:v>两只都装；不能用跳线短接代替。</x:v>
       </x:c>
       <x:c r="J13" s="26"/>
       <x:c r="K13" s="27"/>
@@ -902,7 +902,7 @@
         <x:v>待核对</x:v>
       </x:c>
       <x:c r="M13" s="24" t="str">
-        <x:v>暂停安装，驱动定型后确认新阻值。</x:v>
+        <x:v>现有1kΩ中另取2只。</x:v>
       </x:c>
       <x:c r="N13" s="2"/>
       <x:c r="O13" s="5" t="str">
@@ -1038,29 +1038,28 @@
         <x:v>C10</x:v>
       </x:c>
       <x:c r="B17" s="24" t="str">
-        <x:v>现有无源蜂鸣器（未接线）</x:v>
+        <x:v>现有无源蜂鸣器（驱动采购后试接）</x:v>
       </x:c>
       <x:c r="C17" s="29" t="str">
-        <x:v>型号未知（无源、16Ω已确认）</x:v>
+        <x:v>商品图标3–12V、16Ω；厂家型号未知</x:v>
       </x:c>
       <x:c r="D17" s="24" t="str">
-        <x:v>用户2026-10-17确认：无源、16Ω。额定电压/电流及端子定义待确认。
-用于比赛按键发声和旋律演奏，当前未安装。</x:v>
+        <x:v>直径12mm、高8mm、脚距6mm。基础按键声和指定旋律使用，不必另加扬声器。额定电流待测。</x:v>
       </x:c>
       <x:c r="E17" s="25" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="F17" s="24" t="str">
-        <x:v>个（当前安装）</x:v>
+        <x:v>个（计划）</x:v>
       </x:c>
       <x:c r="G17" s="24" t="str">
-        <x:v>两版共用，声音待设计</x:v>
+        <x:v>两版限流试接共用</x:v>
       </x:c>
       <x:c r="H17" s="24" t="str">
-        <x:v>已有1个无源蜂鸣器，16Ω。2026-10-17用户确认，具体型号未知。</x:v>
+        <x:v>已有1个；3–12V/16Ω依据用户商品图，尚未实测。</x:v>
       </x:c>
       <x:c r="I17" s="24" t="str">
-        <x:v>核对完整型号、额定电压/电流、实物端子定义及脚距；禁止直接接GPIO。</x:v>
+        <x:v>认清实物＋号；禁止直接接PB0。</x:v>
       </x:c>
       <x:c r="J17" s="26"/>
       <x:c r="K17" s="27"/>
@@ -1068,11 +1067,11 @@
         <x:v>待核对</x:v>
       </x:c>
       <x:c r="M17" s="24" t="str">
-        <x:v>已有1个保留待装；待额定参数和三极管型号、脚序确认后设计接线，不补购未知型号。</x:v>
+        <x:v>沿用现有件，驱动采购后先限流试音，音量未验收。</x:v>
       </x:c>
       <x:c r="N17" s="2"/>
       <x:c r="O17" s="5" t="str">
-        <x:v>用户2026-10-17确认：无源蜂鸣器，16Ω；具体型号和额定参数未提供。</x:v>
+        <x:v>用户2026-10-18商品图：3–12V、16Ω、12×8mm、脚距6mm。</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="54" customHeight="1">
@@ -1080,28 +1079,28 @@
         <x:v>C11</x:v>
       </x:c>
       <x:c r="B18" s="5" t="str">
-        <x:v>现有三极管（未接线）</x:v>
+        <x:v>SS8050D直插NPN三极管（待购）</x:v>
       </x:c>
       <x:c r="C18" s="28" t="str">
-        <x:v>用户已有，型号稍后提供</x:v>
+        <x:v>onsemi SS8050DBU / S8050D；TO-92</x:v>
       </x:c>
       <x:c r="D18" s="5" t="str">
-        <x:v>已有三极管，型号稍后提供。器件类型、封装、额定及B/C/E脚序待核对，不能假定NPN/PNP/TO-92；目前未接线。</x:v>
+        <x:v>参考厂家脚序：1=E发射极，2=B基极，3=C集电极。其他品牌须按实际数据表核对。</x:v>
       </x:c>
       <x:c r="E18" s="18" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="F18" s="5" t="str">
-        <x:v>个（当前安装）</x:v>
+        <x:v>个（计划）</x:v>
       </x:c>
       <x:c r="G18" s="5" t="str">
-        <x:v>两版共用，驱动待设计</x:v>
+        <x:v>两版声音试接共用</x:v>
       </x:c>
       <x:c r="H18" s="5" t="str">
-        <x:v>已有三极管，型号稍后提供、数量待清点；没有MOS预焊板。</x:v>
+        <x:v>用户已更正：没有三极管，准备购买；没有MOS转接板。</x:v>
       </x:c>
       <x:c r="I18" s="5" t="str">
-        <x:v>提供完整型号和厂家信息，核对类型、额定值及真实B/C/E脚序；不能套用旧G/D/S。</x:v>
+        <x:v>买直插TO-92 NPN，勿买SS8550或贴片版；核对实际E/B/C。</x:v>
       </x:c>
       <x:c r="J18" s="21"/>
       <x:c r="K18" s="22"/>
@@ -1109,11 +1108,11 @@
         <x:v>待核对</x:v>
       </x:c>
       <x:c r="M18" s="5" t="str">
-        <x:v>先核对现物型号及适用性，不要求AO3400A预焊板。</x:v>
+        <x:v>购买1只，可另备1只；不用MOS预焊转接板。</x:v>
       </x:c>
       <x:c r="N18" s="2"/>
       <x:c r="O18" s="5" t="str">
-        <x:v>用户2026-10-17确认回复</x:v>
+        <x:v>https://www.onsemi.com/download/data-sheet/pdf/ss8050-d.pdf</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="54" customHeight="1">
@@ -1121,29 +1120,28 @@
         <x:v>C12</x:v>
       </x:c>
       <x:c r="B19" s="24" t="str">
-        <x:v>待定的声音驱动下拉电阻</x:v>
+        <x:v>基极下拉电阻</x:v>
       </x:c>
       <x:c r="C19" s="29" t="str">
-        <x:v>旧候选100kΩ；当前不安装</x:v>
+        <x:v>10kΩ（103）轴向直插，≥1/4W</x:v>
       </x:c>
       <x:c r="D19" s="24" t="str">
-        <x:v>旧MOS方案采用100kΩ下拉；三极管驱动定型后重新确定。
-新声音支路设计后确定。</x:v>
+        <x:v>接SS8050D的B与E之间，复位时关闭声音。</x:v>
       </x:c>
       <x:c r="E19" s="25" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="F19" s="24" t="str">
-        <x:v>只（当前安装）</x:v>
+        <x:v>只（计划）</x:v>
       </x:c>
       <x:c r="G19" s="24" t="str">
-        <x:v>两版当前均暂停</x:v>
+        <x:v>两版声音试接共用</x:v>
       </x:c>
       <x:c r="H19" s="24" t="str">
-        <x:v>未确认；用户仅明确有1kΩ和10kΩ</x:v>
+        <x:v>用户有10kΩ，另取1只；按键仍用6只。</x:v>
       </x:c>
       <x:c r="I19" s="24" t="str">
-        <x:v>当前0表示暂不安装；比赛最终仍需声音及相应保护。</x:v>
+        <x:v>不能沿用旧MOS方案的100kΩ值。</x:v>
       </x:c>
       <x:c r="J19" s="26"/>
       <x:c r="K19" s="27"/>
@@ -1151,7 +1149,7 @@
         <x:v>待核对</x:v>
       </x:c>
       <x:c r="M19" s="24" t="str">
-        <x:v>暂停安装，不按旧候选值默认购买。</x:v>
+        <x:v>合计至少7只10kΩ（按键6＋声音1）。</x:v>
       </x:c>
       <x:c r="N19" s="2"/>
       <x:c r="O19" s="5" t="str">
@@ -1163,29 +1161,28 @@
         <x:v>C13</x:v>
       </x:c>
       <x:c r="B20" s="5" t="str">
-        <x:v>待定的声音限流功率电阻</x:v>
+        <x:v>声音试接限流功率电阻（待购）</x:v>
       </x:c>
       <x:c r="C20" s="28" t="str">
-        <x:v>旧候选68Ω、≥1W；当前不安装</x:v>
+        <x:v>47Ω，≥1W，轴向直插</x:v>
       </x:c>
       <x:c r="D20" s="5" t="str">
-        <x:v>需按现有蜂鸣器额定参数和实测供电重定，不默认保留68Ω。
-新声音支路设计后确定。</x:v>
+        <x:v>板上5V经此电阻到蜂鸣器＋。这是初次试接值，可能降低音量；正式值待实测。</x:v>
       </x:c>
       <x:c r="E20" s="18" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="F20" s="5" t="str">
-        <x:v>只（当前安装）</x:v>
+        <x:v>只（计划）</x:v>
       </x:c>
       <x:c r="G20" s="5" t="str">
-        <x:v>两版当前均暂停</x:v>
+        <x:v>两版声音试接共用</x:v>
       </x:c>
       <x:c r="H20" s="5" t="str">
         <x:v>未确认</x:v>
       </x:c>
       <x:c r="I20" s="5" t="str">
-        <x:v>当前0表示暂不安装；比赛最终仍需声音及相应保护。</x:v>
+        <x:v>不拿1/4W普通电阻代替；不能未经测量直接短接。</x:v>
       </x:c>
       <x:c r="J20" s="21"/>
       <x:c r="K20" s="22"/>
@@ -1193,7 +1190,7 @@
         <x:v>待核对</x:v>
       </x:c>
       <x:c r="M20" s="5" t="str">
-        <x:v>暂停安装，不按旧候选值默认购买。</x:v>
+        <x:v>购买1只；先限流试接，测电流、压降与音量。</x:v>
       </x:c>
       <x:c r="N20" s="2"/>
       <x:c r="O20" s="5" t="str">
@@ -1205,29 +1202,28 @@
         <x:v>C14</x:v>
       </x:c>
       <x:c r="B21" s="5" t="str">
-        <x:v>待定的声音保护二极管</x:v>
+        <x:v>蜂鸣器保护二极管</x:v>
       </x:c>
       <x:c r="C21" s="28" t="str">
-        <x:v>旧候选1N5819；当前不安装</x:v>
+        <x:v>1N5819，DO-41直插</x:v>
       </x:c>
       <x:c r="D21" s="5" t="str">
-        <x:v>用户有二极管但型号未知。蜂鸣器已确认无源、16Ω；额定参数和三极管驱动确定后，再定保护器件。
-新声音支路设计后确定。</x:v>
+        <x:v>色环K接蜂鸣器＋；无环A接蜂鸣器−/三极管C。</x:v>
       </x:c>
       <x:c r="E21" s="18" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="F21" s="5" t="str">
-        <x:v>只（当前安装）</x:v>
+        <x:v>只（计划）</x:v>
       </x:c>
       <x:c r="G21" s="5" t="str">
-        <x:v>两版当前均暂停</x:v>
+        <x:v>两版声音试接共用</x:v>
       </x:c>
       <x:c r="H21" s="5" t="str">
         <x:v>用户说有二极管；具体型号与数量未知</x:v>
       </x:c>
       <x:c r="I21" s="5" t="str">
-        <x:v>当前0表示暂不安装；比赛最终仍需声音及相应保护。</x:v>
+        <x:v>现有二极管型号未知；不能凭外形代用。</x:v>
       </x:c>
       <x:c r="J21" s="21"/>
       <x:c r="K21" s="22"/>
@@ -1235,12 +1231,11 @@
         <x:v>待核对</x:v>
       </x:c>
       <x:c r="M21" s="5" t="str">
-        <x:v>暂停安装，不按旧候选值默认购买。</x:v>
+        <x:v>先找1N5819；现有不能确认就补购1只。</x:v>
       </x:c>
       <x:c r="N21" s="2"/>
       <x:c r="O21" s="5" t="str">
-        <x:v>旧声音候选参考，当前不安装。
-https://www.vishay.com/docs/88525/1n5817.pdf</x:v>
+        <x:v>https://www.vishay.com/docs/88525/1n5817.pdf</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="54" customHeight="1">
@@ -1278,7 +1273,7 @@
         <x:v>待核对</x:v>
       </x:c>
       <x:c r="M22" s="5" t="str">
-        <x:v>暂停安装，不按旧候选值默认购买。</x:v>
+        <x:v>可备100nF/16V作去耦；本次试接模型未安装。</x:v>
       </x:c>
       <x:c r="N22" s="2"/>
       <x:c r="O22" s="5" t="str">
@@ -1320,7 +1315,7 @@
         <x:v>待核对</x:v>
       </x:c>
       <x:c r="M23" s="5" t="str">
-        <x:v>暂停安装，不按旧候选值默认购买。</x:v>
+        <x:v>可备100µF/16V作去耦；本次试接模型未安装。</x:v>
       </x:c>
       <x:c r="N23" s="2"/>
       <x:c r="O23" s="5" t="str">
@@ -1587,8 +1582,7 @@
         <x:v>MB-102；用户照片同型两块</x:v>
       </x:c>
       <x:c r="D30" s="24" t="str">
-        <x:v>每块中央a～j、编号1～63。当前只从电源条前半段取电，不装中点桥接。
-第一块轨1/2、控制与OLED，第二块轨3/4；声音配套暂停。</x:v>
+        <x:v>两块MB-102，每块A～J/1～63；电源只用左侧前25孔。按键跨沟槽并错开放置，第二块下端为SS8050D声音试接区。</x:v>
       </x:c>
       <x:c r="E30" s="25" t="n">
         <x:v>2</x:v>
@@ -1629,11 +1623,10 @@
         <x:v>2.54mm公对公杜邦线或适配面包板的实芯短跳线</x:v>
       </x:c>
       <x:c r="D31" s="5" t="str">
-        <x:v>两端金属针。当前29根，可选I²C上拉另加2根；不含旧声音线和5根已撤桥线。
-板内信号、公共地和两板电源连接，电源条只取前半段。</x:v>
+        <x:v>32根公公跳线，含声音支路3根；可选I²C上拉另加2根。电源条不跨中点。</x:v>
       </x:c>
       <x:c r="E31" s="18" t="n">
-        <x:v>29</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="F31" s="5" t="str">
         <x:v>根（当前计划）</x:v>
@@ -1671,11 +1664,10 @@
         <x:v>2.54mm公对母，长度按核心板到面包板／模块距离</x:v>
       </x:c>
       <x:c r="D32" s="5" t="str">
-        <x:v>一端金属针、另一端插孔。核心板23根加OLED4根，共27根，已排除声音支路。
-核心板排针／OLED排针连接面包板。</x:v>
+        <x:v>31根公母线：原核心板与OLED27根，声音控制/取电2根、蜂鸣器脚转接2根。需按实物端子适配。</x:v>
       </x:c>
       <x:c r="E32" s="18" t="n">
-        <x:v>27</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="F32" s="5" t="str">
         <x:v>根（当前计划）</x:v>
@@ -1759,7 +1751,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc321b6af3ec54baf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8681e514b9bd45da"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1807,7 +1799,7 @@
     </x:row>
     <x:row r="2" ht="30" customHeight="1">
       <x:c r="A2" s="3" t="str">
-        <x:v>节奏大师工具、线材与选件（2026-10-17）</x:v>
+        <x:v>节奏大师工具与线材核对（2026-10-18）</x:v>
       </x:c>
       <x:c r="B2" s="2"/>
       <x:c r="C2" s="2"/>
@@ -1864,7 +1856,7 @@
     </x:row>
     <x:row r="5" ht="24" customHeight="1">
       <x:c r="A5" s="2" t="str">
-        <x:v>两版可轮流使用一套通用元件。已有三极管和蜂鸣器型号待核对，旧MOS预焊板方案已停用。</x:v>
+        <x:v>两版可轮流使用一套元件。SS8050D准备采购，无源16Ω蜂鸣器沿用现有件。</x:v>
       </x:c>
       <x:c r="B5" s="2"/>
       <x:c r="C5" s="2"/>
@@ -1883,7 +1875,7 @@
     </x:row>
     <x:row r="6" ht="24" customHeight="1">
       <x:c r="A6" s="2" t="str">
-        <x:v>当前公公29根、公母27根及成品线1条；可选上拉另加2根公公。W03汇总P02～P04、W01，不重复备料。</x:v>
+        <x:v>当前公公32根、公母31根及成品线1条；可选上拉另加2根公公。W03汇总P02～P04、W01。</x:v>
       </x:c>
       <x:c r="B6" s="2"/>
       <x:c r="C6" s="2"/>
@@ -2020,7 +2012,7 @@
         <x:v>待核对</x:v>
       </x:c>
       <x:c r="M9" s="5" t="str">
-        <x:v>按13灯信号、6键信号、3V3/GND及OLED接头清点；声音接口暂不计入。</x:v>
+        <x:v>原信号连接照旧；声音支路采用焊接接线，若要可拆需另配匹配接头。</x:v>
       </x:c>
       <x:c r="N9" s="2"/>
       <x:c r="O9" s="5" t="str">
@@ -2455,7 +2447,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4acc825996db4c8f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8630505d966d434e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Label all resistors, use 330 ohm LED resistors and publish hardware checklist
</commit_message>
<xml_diff>
--- a/hardware-checklist.xlsx
+++ b/hardware-checklist.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="元件核对" sheetId="1" r:id="R3f529c4e737747b3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="工具线材" sheetId="2" r:id="Re31429ef414b4ef6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="元件核对" sheetId="1" r:id="R3f19e5c86e1f4331"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="工具线材" sheetId="2" r:id="Rcc016d4cb1ff4e3a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -596,7 +596,7 @@
     </x:row>
     <x:row r="6" ht="24" customHeight="1">
       <x:c r="A6" s="2" t="str">
-        <x:v>13盏LED、6个按键、OLED与充电宝供电；新增SS8050D限流试接支路，正式声音参数待测。</x:v>
+        <x:v>13灯各串330Ω、6键各10kΩ上拉；声音仍为两只1kΩ并联、10kΩ下拉和47Ω限流。</x:v>
       </x:c>
       <x:c r="B6" s="2"/>
       <x:c r="C6" s="2"/>
@@ -835,10 +835,10 @@
         <x:v>LED限流电阻</x:v>
       </x:c>
       <x:c r="C12" s="28" t="str">
-        <x:v>通用轴向直插1kΩ；厂家及系列不限，现有型号未知</x:v>
+        <x:v>330Ω轴向直插电阻；≥1/4W</x:v>
       </x:c>
       <x:c r="D12" s="5" t="str">
-        <x:v>1kΩ（102），≥1/4W。每盏LED串联1只，本次共13只；声音电阻另行设计。</x:v>
+        <x:v>13颗LED每颗独立串联一只330Ω。四环：橙、橙、棕、金（±5%）。孔位不变。</x:v>
       </x:c>
       <x:c r="E12" s="18" t="n">
         <x:v>13</x:v>
@@ -850,10 +850,10 @@
         <x:v>洞洞板、面包板共用</x:v>
       </x:c>
       <x:c r="H12" s="5" t="str">
-        <x:v>用户确认有1kΩ；数量、功率及精度未知</x:v>
+        <x:v>用户2026-10-18确认：仅LED限流采用330Ω；数量与功率待核对。</x:v>
       </x:c>
       <x:c r="I12" s="5" t="str">
-        <x:v>核对阻值和数量；不能13灯共用1只。</x:v>
+        <x:v>LED电阻用330Ω，不用于替换声音基极或10kΩ上拉。</x:v>
       </x:c>
       <x:c r="J12" s="21"/>
       <x:c r="K12" s="22"/>
@@ -861,7 +861,7 @@
         <x:v>待核对</x:v>
       </x:c>
       <x:c r="M12" s="5" t="str">
-        <x:v>LED用13只；声音基极另用2只1kΩ，合计至少15只。</x:v>
+        <x:v>330Ω共13只；声音基极仍另用1kΩ两只。</x:v>
       </x:c>
       <x:c r="N12" s="2"/>
       <x:c r="O12" s="5" t="str">
@@ -1751,7 +1751,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8681e514b9bd45da"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R343c606a722f42fc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2447,7 +2447,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8630505d966d434e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3adb7f5a29054bc8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>